<commit_message>
🚀 Major Enhancement: Complete LISP & Bridge Integration...
</commit_message>
<xml_diff>
--- a/uploads/input.xlsx
+++ b/uploads/input.xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rajkumar\RajLisp\Tested_Bridge_GAD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rajkumar\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25125" windowHeight="12315"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="111">
   <si>
     <t>Abutment Left Cap Width Excluding D/W</t>
   </si>
@@ -190,6 +190,12 @@
     <t>Read Chainage Of Left Abutment TO BE INCRESED FOR COMPLETE DRAWING OF APPROACH</t>
   </si>
   <si>
+    <t>Abt Left Front Batter ( 1 HOR : 10 VER &gt;&gt;&gt;&gt;&gt; VALUE 10)</t>
+  </si>
+  <si>
+    <t>Abt Left  Toe Batter ( 1 HOR : 5 VER &gt;&gt;&gt;&gt;&gt; VALUE 5)</t>
+  </si>
+  <si>
     <t>Abutment RIGHT Footing Level</t>
   </si>
   <si>
@@ -362,21 +368,6 @@
   </si>
   <si>
     <t xml:space="preserve">Scale1 </t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Variable</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Abt Left Front Batter ( e.g. 1 HOR : 10 VER &gt;&gt;&gt;&gt;&gt; VALUE 10)</t>
-  </si>
-  <si>
-    <t>Abt Left  Toe Batter (e.g.  1 HOR : 5 VER &gt;&gt;&gt;&gt;&gt; VALUE 5)</t>
   </si>
 </sst>
 </file>
@@ -483,7 +474,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -527,11 +518,6 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -849,7 +835,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -858,565 +844,565 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
-        <v>109</v>
-      </c>
-      <c r="B1" s="26" t="s">
+      <c r="A1" s="7">
+        <v>186</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="C1" s="27" t="s">
-        <v>111</v>
-      </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="19">
+      <c r="A2" s="10">
+        <f>A44</f>
+        <v>12</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="10">
+        <v>0.3</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="10">
+        <v>0.75</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="11">
-        <f>A2+(A5*A6)</f>
-        <v>388.8</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="20">
-        <v>21</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>8</v>
-      </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="20">
-        <v>36</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>22</v>
+      <c r="A5" s="12">
+        <f>IF(Sheet3!B2+2&gt;(A31-2),A31-5,Sheet3!B2+2)</f>
+        <v>100</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="10">
-        <v>10.8</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>14</v>
+      <c r="A6" s="12">
+        <f>A5+0.75</f>
+        <v>100.75</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="12">
-        <f>A3-A2</f>
-        <v>388.8</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>38</v>
+      <c r="A7" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="7">
-        <v>186</v>
+      <c r="A8" s="16">
+        <v>10</v>
       </c>
       <c r="B8" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="12">
+        <f>A5+A15</f>
+        <v>101</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="12">
+        <f>A6</f>
+        <v>100.75</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10" s="14" t="s">
         <v>54</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="10">
-        <f>A46</f>
-        <v>12</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="10">
-        <v>0.3</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="10">
-        <v>0.75</v>
+        <v>10</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>0</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="12">
-        <f>IF(Sheet3!B2+2&gt;(A33-2),A33-5,Sheet3!B2+2)</f>
-        <v>100</v>
+        <f>A5+A15</f>
+        <v>101</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>48</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="12">
-        <f>A12+0.75</f>
+        <f>A10</f>
         <v>100.75</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="10">
-        <v>1.2</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="C14" s="9" t="s">
+      <c r="A14" s="16">
+        <v>1.5</v>
+      </c>
+      <c r="B14" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="16">
-        <v>10</v>
-      </c>
       <c r="B15" s="8" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>112</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="12">
-        <f>A12+A22</f>
-        <v>101</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>49</v>
+      <c r="A16" s="16">
+        <v>3</v>
+      </c>
+      <c r="B16" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="12">
-        <f>A13</f>
+        <f>A9</f>
+        <v>101</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="12">
+        <f>A10</f>
         <v>100.75</v>
       </c>
-      <c r="B17" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="10">
-        <v>10</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>113</v>
+      <c r="B18" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="12">
-        <f>A12+A22</f>
-        <v>101</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="C19" s="14" t="s">
-        <v>2</v>
+      <c r="A19" s="7">
+        <v>100</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="12">
-        <f>A17</f>
-        <v>100.75</v>
-      </c>
-      <c r="B20" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>53</v>
+      <c r="A20" s="21">
+        <v>0</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="C20" s="23" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="16">
-        <v>1.5</v>
-      </c>
-      <c r="B21" s="24" t="s">
-        <v>67</v>
-      </c>
-      <c r="C21" s="15" t="s">
-        <v>33</v>
+      <c r="A21" s="10">
+        <v>100</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="10">
+        <v>110.97499999999999</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="19">
+        <v>0</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="11">
+        <f>A23+(A28*A46)</f>
+        <v>97.2</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="10">
+        <v>10</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="10">
         <v>1</v>
       </c>
-      <c r="B22" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="16">
-        <v>3</v>
-      </c>
-      <c r="B23" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="12">
-        <f>A16</f>
-        <v>101</v>
-      </c>
-      <c r="B24" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="12">
-        <f>A17</f>
-        <v>100.75</v>
-      </c>
-      <c r="B25" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="7">
-        <v>100</v>
-      </c>
       <c r="B26" s="8" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>36</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="21">
+      <c r="A27" s="20">
+        <v>21</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="20">
+        <v>9</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="12">
+        <f>A24-A23</f>
+        <v>97.2</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C29" s="14" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="16">
         <v>0</v>
       </c>
-      <c r="B27" s="22" t="s">
-        <v>73</v>
-      </c>
-      <c r="C27" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="10">
-        <v>100</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="10">
-        <v>110.97499999999999</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C29" s="9" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="10">
-        <v>10</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>6</v>
+      <c r="B30" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="10">
-        <v>1</v>
+        <f>A22</f>
+        <v>110.97499999999999</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="16">
-        <v>0</v>
-      </c>
-      <c r="B32" s="24" t="s">
-        <v>83</v>
-      </c>
-      <c r="C32" s="15" t="s">
-        <v>50</v>
+      <c r="A32" s="10">
+        <v>110</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="10">
-        <f>A29</f>
-        <v>110.97499999999999</v>
+        <v>0.22500000000000001</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="10">
-        <v>110</v>
+        <v>0.22500000000000001</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>9</v>
+        <v>40</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="10">
-        <v>0.22500000000000001</v>
+        <v>11.1</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="10">
-        <v>0.22500000000000001</v>
+        <v>0.9</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="10">
-        <v>11.1</v>
+        <v>0.75</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="10">
-        <v>0.9</v>
+        <v>0.75</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="10">
-        <v>0.75</v>
+        <v>110</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>43</v>
+        <v>105</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="10">
-        <v>0.75</v>
+        <v>109.4</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>44</v>
+        <v>106</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="10">
-        <v>110</v>
+        <v>1.2</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>103</v>
+        <v>45</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="10">
-        <v>109.4</v>
+        <v>1.2</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>104</v>
+        <v>11</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="10">
-        <v>1.2</v>
+      <c r="A43" s="16">
+        <v>10</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="C43" s="9" t="s">
-        <v>45</v>
+        <v>98</v>
+      </c>
+      <c r="C43" s="15" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="10">
-        <v>1.2</v>
+        <v>12</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="16">
-        <v>10</v>
+      <c r="A45" s="10">
+        <v>1</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="C45" s="15" t="s">
-        <v>12</v>
+        <v>100</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="10">
-        <v>12</v>
+        <v>10.8</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>97</v>
+        <v>17</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="10">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>98</v>
+        <v>18</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>46</v>
+        <v>24</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="10">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="10">
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="10">
-        <v>4.5</v>
+        <v>12</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>47</v>
+        <v>16</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1424,65 +1410,54 @@
         <v>12</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="10">
-        <v>12</v>
+        <v>3.5</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>55</v>
+        <v>101</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="10">
-        <v>3.5</v>
+        <f>12</f>
+        <v>12</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="10">
-        <f>12</f>
-        <v>12</v>
+        <v>0.375</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="10">
-        <v>0.375</v>
+        <v>7.4999999999999997E-2</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="10">
-        <v>7.4999999999999997E-2</v>
-      </c>
-      <c r="B56" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="C56" s="9" t="s">
         <v>30</v>
       </c>
     </row>

</xml_diff>